<commit_message>
updated figure order, generated source data
</commit_message>
<xml_diff>
--- a/outputdir/EDTable_14_OR_invasiveness.xlsx
+++ b/outputdir/EDTable_14_OR_invasiveness.xlsx
@@ -12,9 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count</t>
   </si>
   <si>
     <t xml:space="preserve">std_error</t>
@@ -446,465 +449,537 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0254051284671005</v>
+        <v>577</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0485601350235334</v>
+        <v>0.26585435624863</v>
       </c>
       <c r="D2" t="n">
-        <v>1.05140026525965</v>
+        <v>0.103821071707496</v>
       </c>
       <c r="E2" t="n">
-        <v>1.00032886396341</v>
+        <v>1.54101294449123</v>
       </c>
       <c r="F2" t="n">
-        <v>1.10507909709631</v>
+        <v>0.91517993580637</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.59481310961777</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0498106200925398</v>
+        <v>70</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0783510066582239</v>
+        <v>0.495865001221417</v>
       </c>
       <c r="D3" t="n">
-        <v>1.09166314044835</v>
+        <v>0.101698240548849</v>
       </c>
       <c r="E3" t="n">
-        <v>0.990122639650321</v>
+        <v>2.2514404648926</v>
       </c>
       <c r="F3" t="n">
-        <v>1.20361697075672</v>
+        <v>0.851866730146506</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.95044270138834</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0721759329795116</v>
+        <v>23</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0260969472257768</v>
+        <v>0.648854424824996</v>
       </c>
       <c r="D4" t="n">
-        <v>1.17424453282037</v>
+        <v>0.0550097121601589</v>
       </c>
       <c r="E4" t="n">
-        <v>1.01934489523295</v>
+        <v>3.47300964572325</v>
       </c>
       <c r="F4" t="n">
-        <v>1.35268271740687</v>
+        <v>0.973621045327573</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12.3885941631722</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0696212303196379</v>
+        <v>24</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00965234469503171</v>
+        <v>0.619375300761202</v>
       </c>
       <c r="D5" t="n">
-        <v>1.19752367968121</v>
+        <v>0.0285957093958869</v>
       </c>
       <c r="E5" t="n">
-        <v>1.04477151224989</v>
+        <v>3.87994961715428</v>
       </c>
       <c r="F5" t="n">
-        <v>1.3726091749085</v>
+        <v>1.1523998323963</v>
+      </c>
+      <c r="G5" t="n">
+        <v>13.0631822466968</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0525025675160563</v>
+        <v>47</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00682484856218778</v>
+        <v>0.511523575478637</v>
       </c>
       <c r="D6" t="n">
-        <v>0.867537888767302</v>
+        <v>0.0164532804466746</v>
       </c>
       <c r="E6" t="n">
-        <v>0.782703657986305</v>
+        <v>0.293172873753352</v>
       </c>
       <c r="F6" t="n">
-        <v>0.96156697463652</v>
+        <v>0.10757370493122</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.79899018035823</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="n">
-        <v>0.0796147633874422</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>0.00966687624140562</v>
+        <v>0.651048842350722</v>
       </c>
       <c r="D7" t="n">
-        <v>1.22886220396691</v>
+        <v>0.1180855281828</v>
       </c>
       <c r="E7" t="n">
-        <v>1.05131710900474</v>
+        <v>2.76626543695553</v>
       </c>
       <c r="F7" t="n">
-        <v>1.43639088853791</v>
+        <v>0.772164600827542</v>
+      </c>
+      <c r="G7" t="n">
+        <v>9.91009489361951</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0791570726945935</v>
+        <v>18</v>
       </c>
       <c r="C8" t="n">
-        <v>0.144189310820879</v>
+        <v>0.757179547970182</v>
       </c>
       <c r="D8" t="n">
-        <v>1.12256637087014</v>
+        <v>0.209617104426024</v>
       </c>
       <c r="E8" t="n">
-        <v>0.961240735796996</v>
+        <v>2.58563685661161</v>
       </c>
       <c r="F8" t="n">
-        <v>1.31096738837615</v>
+        <v>0.586196588616131</v>
+      </c>
+      <c r="G8" t="n">
+        <v>11.4049076437843</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" t="n">
-        <v>0.104156539834331</v>
+        <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>0.00904441206682928</v>
+        <v>0.989238174556678</v>
       </c>
       <c r="D9" t="n">
-        <v>1.31258613215891</v>
+        <v>0.031977987895949</v>
       </c>
       <c r="E9" t="n">
-        <v>1.07020746238305</v>
+        <v>8.3445191247445</v>
       </c>
       <c r="F9" t="n">
-        <v>1.60985828906435</v>
+        <v>1.20045194769182</v>
+      </c>
+      <c r="G9" t="n">
+        <v>58.0039872125747</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10" t="n">
-        <v>0.0853179357332782</v>
+        <v>26</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0000516599525591779</v>
+        <v>0.876551820257151</v>
       </c>
       <c r="D10" t="n">
-        <v>1.41295465050329</v>
+        <v>0.0100184865105537</v>
       </c>
       <c r="E10" t="n">
-        <v>1.19537489359376</v>
+        <v>9.55713501881229</v>
       </c>
       <c r="F10" t="n">
-        <v>1.67013784134013</v>
+        <v>1.71471421838166</v>
+      </c>
+      <c r="G10" t="n">
+        <v>53.2676692061335</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11" t="n">
-        <v>0.0729445907091588</v>
+        <v>26</v>
       </c>
       <c r="C11" t="n">
-        <v>0.000312971978032461</v>
+        <v>0.7263613163475</v>
       </c>
       <c r="D11" t="n">
-        <v>1.30096959308993</v>
+        <v>0.00600861007504854</v>
       </c>
       <c r="E11" t="n">
-        <v>1.12765294122504</v>
+        <v>7.3561782964014</v>
       </c>
       <c r="F11" t="n">
-        <v>1.50092446023853</v>
+        <v>1.7715809936115</v>
+      </c>
+      <c r="G11" t="n">
+        <v>30.5452357660109</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12" t="n">
-        <v>0.0369817952932345</v>
+        <v>123</v>
       </c>
       <c r="C12" t="n">
-        <v>0.00021670237113267</v>
+        <v>0.32647318244589</v>
       </c>
       <c r="D12" t="n">
-        <v>1.14670289415024</v>
+        <v>0.00238032625156854</v>
       </c>
       <c r="E12" t="n">
-        <v>1.06652580774566</v>
+        <v>2.69628705348856</v>
       </c>
       <c r="F12" t="n">
-        <v>1.23290736886334</v>
+        <v>1.4218917789021</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5.11288129144642</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B13" t="n">
-        <v>0.0331563249045609</v>
+        <v>132</v>
       </c>
       <c r="C13" t="n">
-        <v>0.000096729492731968</v>
+        <v>0.292710516088035</v>
       </c>
       <c r="D13" t="n">
-        <v>1.13811747824334</v>
+        <v>0.0143478264955189</v>
       </c>
       <c r="E13" t="n">
-        <v>1.0665073661635</v>
+        <v>2.04762935055936</v>
       </c>
       <c r="F13" t="n">
-        <v>1.21453581604649</v>
+        <v>1.15369530346109</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3.63422295704402</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B14" t="n">
-        <v>0.0857388391602146</v>
+        <v>16</v>
       </c>
       <c r="C14" t="n">
-        <v>0.315630913820523</v>
+        <v>0.721315437104047</v>
       </c>
       <c r="D14" t="n">
-        <v>1.08985650344134</v>
+        <v>0.329340910138331</v>
       </c>
       <c r="E14" t="n">
-        <v>0.92127003747937</v>
+        <v>2.02101849270301</v>
       </c>
       <c r="F14" t="n">
-        <v>1.28929320369869</v>
+        <v>0.49155734730119</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8.30933719183098</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B15" t="n">
-        <v>0.0592393863792702</v>
+        <v>44</v>
       </c>
       <c r="C15" t="n">
-        <v>0.753546338010647</v>
+        <v>0.622846327942864</v>
       </c>
       <c r="D15" t="n">
-        <v>0.981571645287802</v>
+        <v>0.703077630952566</v>
       </c>
       <c r="E15" t="n">
-        <v>0.873969789665046</v>
+        <v>0.788667949841579</v>
       </c>
       <c r="F15" t="n">
-        <v>1.10242128071986</v>
+        <v>0.232657305750058</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2.67344768350204</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B16" t="n">
-        <v>0.0823619837408271</v>
+        <v>27</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0791470277924633</v>
+        <v>0.6909633430299</v>
       </c>
       <c r="D16" t="n">
-        <v>1.15561252785067</v>
+        <v>0.073156381283116</v>
       </c>
       <c r="E16" t="n">
-        <v>0.983341358081759</v>
+        <v>3.4490723872544</v>
       </c>
       <c r="F16" t="n">
-        <v>1.35806381329319</v>
+        <v>0.890312431964176</v>
+      </c>
+      <c r="G16" t="n">
+        <v>13.3617142762749</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17" t="n">
-        <v>0.118727733942215</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
-        <v>0.00696293946709152</v>
+        <v>1.13269982749468</v>
       </c>
       <c r="D17" t="n">
-        <v>1.37787177420224</v>
+        <v>0.0170489278913104</v>
       </c>
       <c r="E17" t="n">
-        <v>1.09180660242577</v>
+        <v>14.9128957553247</v>
       </c>
       <c r="F17" t="n">
-        <v>1.73888912370112</v>
+        <v>1.6195278621975</v>
+      </c>
+      <c r="G17" t="n">
+        <v>137.320551872088</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18" t="n">
-        <v>0.0246468851732945</v>
+        <v>345</v>
       </c>
       <c r="C18" t="n">
-        <v>0.130744876612041</v>
+        <v>0.225694524660532</v>
       </c>
       <c r="D18" t="n">
-        <v>1.03795467040216</v>
+        <v>0.0560965052849797</v>
       </c>
       <c r="E18" t="n">
-        <v>0.989005109263455</v>
+        <v>1.53901238913559</v>
       </c>
       <c r="F18" t="n">
-        <v>1.08932692836339</v>
+        <v>0.98884235011234</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.39528488403005</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B19" t="n">
-        <v>0.0684745286872778</v>
+        <v>26</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0000388726526892239</v>
+        <v>0.550099191460845</v>
       </c>
       <c r="D19" t="n">
-        <v>1.32574739157219</v>
+        <v>0.00464213518939405</v>
       </c>
       <c r="E19" t="n">
-        <v>1.15924194208774</v>
+        <v>4.7458007773236</v>
       </c>
       <c r="F19" t="n">
-        <v>1.51616852569629</v>
+        <v>1.61456531380029</v>
+      </c>
+      <c r="G19" t="n">
+        <v>13.9496524702569</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20" t="n">
-        <v>0.0445370102726884</v>
+        <v>87</v>
       </c>
       <c r="C20" t="n">
-        <v>0.000000000938992534646313</v>
+        <v>0.436001640654009</v>
       </c>
       <c r="D20" t="n">
-        <v>1.31402618307451</v>
+        <v>0.0000121732177514711</v>
       </c>
       <c r="E20" t="n">
-        <v>1.20418538100142</v>
+        <v>6.73469635590964</v>
       </c>
       <c r="F20" t="n">
-        <v>1.43388620809318</v>
+        <v>2.86540444764737</v>
+      </c>
+      <c r="G20" t="n">
+        <v>15.8288771567805</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21" t="n">
-        <v>0.0506203307471061</v>
+        <v>59</v>
       </c>
       <c r="C21" t="n">
-        <v>0.019133715385297</v>
+        <v>0.46178114334131</v>
       </c>
       <c r="D21" t="n">
-        <v>1.12596425073748</v>
+        <v>0.0190521792005937</v>
       </c>
       <c r="E21" t="n">
-        <v>1.01961380397695</v>
+        <v>2.95249267763311</v>
       </c>
       <c r="F21" t="n">
-        <v>1.24340754214376</v>
+        <v>1.1942982185698</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7.29902538238418</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B22" t="n">
-        <v>0.0910472133697177</v>
+        <v>14</v>
       </c>
       <c r="C22" t="n">
-        <v>0.140158697126875</v>
+        <v>0.721575359579764</v>
       </c>
       <c r="D22" t="n">
-        <v>1.14377636810144</v>
+        <v>0.292023756063699</v>
       </c>
       <c r="E22" t="n">
-        <v>0.956841859959564</v>
+        <v>2.13895735654662</v>
       </c>
       <c r="F22" t="n">
-        <v>1.36723155097187</v>
+        <v>0.519977773786653</v>
+      </c>
+      <c r="G22" t="n">
+        <v>8.79871949104135</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B23" t="n">
-        <v>0.0585065117888672</v>
+        <v>38</v>
       </c>
       <c r="C23" t="n">
-        <v>0.198075387790691</v>
+        <v>0.529998665644147</v>
       </c>
       <c r="D23" t="n">
-        <v>1.0782200825181</v>
+        <v>0.499353917960861</v>
       </c>
       <c r="E23" t="n">
-        <v>0.961403432440162</v>
+        <v>1.43049084177547</v>
       </c>
       <c r="F23" t="n">
-        <v>1.20923070078356</v>
+        <v>0.506222110074763</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4.04230476638265</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24" t="n">
-        <v>0.0250555987863459</v>
+        <v>259</v>
       </c>
       <c r="C24" t="n">
-        <v>0.600307598961888</v>
+        <v>0.264435435807944</v>
       </c>
       <c r="D24" t="n">
-        <v>1.01321553321727</v>
+        <v>0.806114633130084</v>
       </c>
       <c r="E24" t="n">
-        <v>0.964659582870891</v>
+        <v>1.06705596144132</v>
       </c>
       <c r="F24" t="n">
-        <v>1.06421553777293</v>
+        <v>0.635470229158608</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1.79175730443742</v>
       </c>
     </row>
   </sheetData>

</xml_diff>